<commit_message>
Import firearm data and filter retired talent maxima
</commit_message>
<xml_diff>
--- a/NN_Feuerwaffen_1.1.xlsx
+++ b/NN_Feuerwaffen_1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Das Western Rollenspiel\LLM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0054FC-1C86-4EDE-8EB3-B110A816513D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFD1666-9BE5-46AB-83B6-1DFE2C760999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="0" windowWidth="26010" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Waffen" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="_FilterDatabase_0" localSheetId="0">Waffen!$A$1:$AE$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Munition!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ressourcen-Waffen'!$A$1:$AI$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Waffen!$A$1:$AE$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Waffen!$A$1:$AG$100</definedName>
     <definedName name="Anpassung">Waffen!$A$91:$A$93</definedName>
     <definedName name="gobherstellung">'Ressourcen-Waffen'!$AL$3:$AL$9</definedName>
     <definedName name="Herstellung">'Ressourcen-Waffen'!$AM$3:$AM$8</definedName>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="381">
   <si>
     <t>Name</t>
   </si>
@@ -1198,6 +1198,9 @@
   </si>
   <si>
     <t>Preis (1.000Schuss)</t>
+  </si>
+  <si>
+    <t>Ini</t>
   </si>
 </sst>
 </file>
@@ -2740,7 +2743,7 @@
     <col min="31" max="1025" width="11.42578125" style="162" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2837,8 +2840,11 @@
       <c r="AF1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG1" s="9" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
         <v>32</v>
       </c>
@@ -2954,11 +2960,14 @@
         <v>589.9</v>
       </c>
       <c r="AF2">
-        <f t="shared" ref="AF2:AF33" si="21">VLOOKUP(AB2,verftab,2,1)</f>
+        <f>VLOOKUP(AB2,verftab,2,1)</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG2" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>41</v>
       </c>
@@ -3074,11 +3083,14 @@
         <v>229.9</v>
       </c>
       <c r="AF3">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="AF2:AF33" si="21">VLOOKUP(AB3,verftab,2,1)</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG3" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>43</v>
       </c>
@@ -3197,8 +3209,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG4" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>45</v>
       </c>
@@ -3317,8 +3332,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG5" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>46</v>
       </c>
@@ -3437,8 +3455,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG6" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>49</v>
       </c>
@@ -3557,8 +3578,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG7" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="s">
         <v>51</v>
       </c>
@@ -3677,8 +3701,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG8" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
         <v>57</v>
       </c>
@@ -3797,8 +3824,11 @@
         <f t="shared" si="21"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG9" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
         <v>62</v>
       </c>
@@ -3917,8 +3947,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG10" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
         <v>63</v>
       </c>
@@ -4037,8 +4070,11 @@
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG11" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>64</v>
       </c>
@@ -4157,8 +4193,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG12" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
         <v>65</v>
       </c>
@@ -4277,8 +4316,11 @@
         <f t="shared" si="21"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG13" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
         <v>67</v>
       </c>
@@ -4397,8 +4439,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG14" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
         <v>68</v>
       </c>
@@ -4517,8 +4562,11 @@
         <f t="shared" si="21"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG15" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" s="35" t="s">
         <v>70</v>
       </c>
@@ -4637,8 +4685,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG16" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" s="35" t="s">
         <v>72</v>
       </c>
@@ -4757,8 +4808,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG17" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" s="35" t="s">
         <v>73</v>
       </c>
@@ -4877,8 +4931,11 @@
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG18" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" s="35" t="s">
         <v>76</v>
       </c>
@@ -4997,8 +5054,11 @@
         <f t="shared" si="21"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG19" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" s="35" t="s">
         <v>78</v>
       </c>
@@ -5117,8 +5177,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG20" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" s="35" t="s">
         <v>79</v>
       </c>
@@ -5237,8 +5300,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG21" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" s="35" t="s">
         <v>81</v>
       </c>
@@ -5357,8 +5423,11 @@
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG22" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" s="35" t="s">
         <v>82</v>
       </c>
@@ -5477,8 +5546,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG23" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" s="35" t="s">
         <v>84</v>
       </c>
@@ -5597,8 +5669,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG24" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" s="35" t="s">
         <v>85</v>
       </c>
@@ -5717,8 +5792,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG25" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A26" s="37" t="s">
         <v>86</v>
       </c>
@@ -5837,8 +5915,11 @@
         <f t="shared" si="21"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG26" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A27" s="37" t="s">
         <v>89</v>
       </c>
@@ -5957,8 +6038,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG27" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A28" s="37" t="s">
         <v>91</v>
       </c>
@@ -6077,8 +6161,11 @@
         <f t="shared" si="21"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG28" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A29" s="37" t="s">
         <v>92</v>
       </c>
@@ -6197,8 +6284,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG29" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A30" s="37" t="s">
         <v>94</v>
       </c>
@@ -6317,8 +6407,11 @@
         <f t="shared" si="21"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG30" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
         <v>95</v>
       </c>
@@ -6437,8 +6530,11 @@
         <f t="shared" si="21"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG31" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
         <v>96</v>
       </c>
@@ -6557,8 +6653,11 @@
         <f t="shared" si="21"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG32" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A33" s="37" t="s">
         <v>98</v>
       </c>
@@ -6677,8 +6776,11 @@
         <f t="shared" si="21"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG33" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
         <v>99</v>
       </c>
@@ -6797,8 +6899,11 @@
         <f t="shared" ref="AF34:AF65" si="43">VLOOKUP(AB34,verftab,2,1)</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG34" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
         <v>100</v>
       </c>
@@ -6917,8 +7022,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG35" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
         <v>101</v>
       </c>
@@ -7037,8 +7145,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG36" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A37" s="37" t="s">
         <v>102</v>
       </c>
@@ -7157,8 +7268,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="38" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG37" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A38" s="37" t="s">
         <v>103</v>
       </c>
@@ -7277,8 +7391,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="39" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG38" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A39" s="37" t="s">
         <v>105</v>
       </c>
@@ -7397,8 +7514,11 @@
         <f t="shared" si="43"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="40" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG39" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
         <v>106</v>
       </c>
@@ -7517,8 +7637,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="41" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG40" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A41" s="37" t="s">
         <v>107</v>
       </c>
@@ -7637,8 +7760,11 @@
         <f t="shared" si="43"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG41" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A42" s="37" t="s">
         <v>110</v>
       </c>
@@ -7757,8 +7883,11 @@
         <f t="shared" si="43"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG42" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A43" s="37" t="s">
         <v>111</v>
       </c>
@@ -7877,8 +8006,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="44" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG43" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A44" s="37" t="s">
         <v>112</v>
       </c>
@@ -7997,8 +8129,11 @@
         <f t="shared" si="43"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="45" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG44" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A45" s="37" t="s">
         <v>113</v>
       </c>
@@ -8117,8 +8252,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="46" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG45" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A46" s="37" t="s">
         <v>114</v>
       </c>
@@ -8237,8 +8375,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="47" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG46" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A47" s="37" t="s">
         <v>115</v>
       </c>
@@ -8357,8 +8498,11 @@
         <f t="shared" si="43"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="48" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG47" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A48" s="37" t="s">
         <v>117</v>
       </c>
@@ -8477,8 +8621,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG48" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A49" s="37" t="s">
         <v>119</v>
       </c>
@@ -8597,8 +8744,11 @@
         <f t="shared" si="43"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="50" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG49" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A50" s="37" t="s">
         <v>120</v>
       </c>
@@ -8717,8 +8867,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="51" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG50" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A51" s="37" t="s">
         <v>121</v>
       </c>
@@ -8837,8 +8990,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="52" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG51" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A52" s="37" t="s">
         <v>123</v>
       </c>
@@ -8957,8 +9113,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="53" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG52" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A53" s="37" t="s">
         <v>124</v>
       </c>
@@ -9077,8 +9236,11 @@
         <f t="shared" si="43"/>
         <v>2</v>
       </c>
-    </row>
-    <row r="54" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG53" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A54" s="37" t="s">
         <v>125</v>
       </c>
@@ -9197,8 +9359,11 @@
         <f t="shared" si="43"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="55" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG54" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A55" s="37" t="s">
         <v>126</v>
       </c>
@@ -9317,8 +9482,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="56" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG55" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A56" s="39" t="s">
         <v>127</v>
       </c>
@@ -9437,8 +9605,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="57" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG56" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A57" s="39" t="s">
         <v>129</v>
       </c>
@@ -9557,8 +9728,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="58" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG57" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A58" s="39" t="s">
         <v>130</v>
       </c>
@@ -9677,8 +9851,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG58" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A59" s="39" t="s">
         <v>131</v>
       </c>
@@ -9797,8 +9974,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="60" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG59" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A60" s="39" t="s">
         <v>132</v>
       </c>
@@ -9917,8 +10097,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="61" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG60" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A61" s="39" t="s">
         <v>133</v>
       </c>
@@ -10037,8 +10220,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="62" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG61" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A62" s="39" t="s">
         <v>134</v>
       </c>
@@ -10157,8 +10343,11 @@
         <f t="shared" si="43"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="63" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG62" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A63" s="39" t="s">
         <v>135</v>
       </c>
@@ -10277,8 +10466,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="64" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG63" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A64" s="39" t="s">
         <v>136</v>
       </c>
@@ -10397,8 +10589,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="65" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG64" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A65" s="39" t="s">
         <v>137</v>
       </c>
@@ -10517,8 +10712,11 @@
         <f t="shared" si="43"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="66" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG65" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A66" s="39" t="s">
         <v>138</v>
       </c>
@@ -10622,7 +10820,7 @@
         <v>70</v>
       </c>
       <c r="AC66" s="28">
-        <f t="shared" ref="AC66:AC97" si="62">VLOOKUP(I66,Res,31,0)*AD66+AE66</f>
+        <f t="shared" ref="AC66:AC87" si="62">VLOOKUP(I66,Res,31,0)*AD66+AE66</f>
         <v>305.55</v>
       </c>
       <c r="AD66" s="29">
@@ -10637,8 +10835,11 @@
         <f t="shared" ref="AF66:AF87" si="65">VLOOKUP(AB66,verftab,2,1)</f>
         <v>6</v>
       </c>
-    </row>
-    <row r="67" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG66" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A67" s="39" t="s">
         <v>139</v>
       </c>
@@ -10757,8 +10958,11 @@
         <f t="shared" si="65"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="68" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG67" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A68" s="39" t="s">
         <v>140</v>
       </c>
@@ -10877,8 +11081,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="69" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG68" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A69" s="41" t="s">
         <v>141</v>
       </c>
@@ -10997,8 +11204,11 @@
         <f t="shared" si="65"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="70" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG69" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A70" s="41" t="s">
         <v>143</v>
       </c>
@@ -11117,8 +11327,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="71" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG70" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A71" s="41" t="s">
         <v>144</v>
       </c>
@@ -11237,8 +11450,11 @@
         <f t="shared" si="65"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="72" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG71" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A72" s="41" t="s">
         <v>145</v>
       </c>
@@ -11357,8 +11573,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="73" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG72" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A73" s="41" t="s">
         <v>146</v>
       </c>
@@ -11477,8 +11696,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="74" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG73" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A74" s="41" t="s">
         <v>147</v>
       </c>
@@ -11597,8 +11819,11 @@
         <f t="shared" si="65"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="75" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG74" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A75" s="41" t="s">
         <v>148</v>
       </c>
@@ -11717,8 +11942,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="76" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG75" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A76" s="41" t="s">
         <v>149</v>
       </c>
@@ -11837,8 +12065,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="77" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG76" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A77" s="41" t="s">
         <v>150</v>
       </c>
@@ -11957,8 +12188,11 @@
         <f t="shared" si="65"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="78" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG77" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A78" s="41" t="s">
         <v>151</v>
       </c>
@@ -12077,8 +12311,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="79" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG78" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A79" s="41" t="s">
         <v>152</v>
       </c>
@@ -12197,8 +12434,11 @@
         <f t="shared" si="65"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="80" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG79" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A80" s="41" t="s">
         <v>153</v>
       </c>
@@ -12317,8 +12557,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="81" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG80" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A81" s="41" t="s">
         <v>154</v>
       </c>
@@ -12437,8 +12680,11 @@
         <f t="shared" si="65"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="82" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG81" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A82" s="41" t="s">
         <v>155</v>
       </c>
@@ -12557,8 +12803,11 @@
         <f t="shared" si="65"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="83" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG82" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A83" s="41" t="s">
         <v>156</v>
       </c>
@@ -12677,8 +12926,11 @@
         <f t="shared" si="65"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="84" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG83" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A84" s="41" t="s">
         <v>157</v>
       </c>
@@ -12797,8 +13049,11 @@
         <f t="shared" si="65"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="85" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG84" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A85" s="41" t="s">
         <v>158</v>
       </c>
@@ -12917,8 +13172,11 @@
         <f t="shared" si="65"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="86" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG85" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A86" s="41" t="s">
         <v>159</v>
       </c>
@@ -13037,8 +13295,11 @@
         <f t="shared" si="65"/>
         <v>7</v>
       </c>
-    </row>
-    <row r="87" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG86" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A87" s="41" t="s">
         <v>160</v>
       </c>
@@ -13157,26 +13418,29 @@
         <f t="shared" si="65"/>
         <v>3</v>
       </c>
-    </row>
-    <row r="90" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG87" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A90" s="16"/>
     </row>
-    <row r="91" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A91" s="161"/>
     </row>
-    <row r="92" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A92" s="161"/>
     </row>
-    <row r="93" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A93" s="161"/>
     </row>
-    <row r="94" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A94" s="161"/>
     </row>
-    <row r="95" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A95" s="161"/>
     </row>
-    <row r="96" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A96" s="161"/>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
@@ -13192,11 +13456,7 @@
       <c r="A100" s="161"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE100" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE100">
-      <sortCondition ref="B1:B100"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:AG100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J87" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>Anpassung</formula1>

</xml_diff>

<commit_message>
Update firearm composition to customize processing and modifications
</commit_message>
<xml_diff>
--- a/NN_Feuerwaffen_1.1.xlsx
+++ b/NN_Feuerwaffen_1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Das Western Rollenspiel\LLM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFD1666-9BE5-46AB-83B6-1DFE2C760999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09394C19-92EE-4C47-82E4-B1B3CD670A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23655" yWindow="525" windowWidth="26010" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Waffen" sheetId="1" r:id="rId1"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="AB2" s="27">
         <f t="shared" ref="AB2:AB33" si="17">VLOOKUP(B2,Res,28,0)+VLOOKUP(C2,Res,28,0)+VLOOKUP(D2,Res,28,0)+VLOOKUP(E2,Res,28,0)+VLOOKUP(F2,Res,28,0)+VLOOKUP(G2,Res,28,0)+VLOOKUP(I2,Res,28,0)+VLOOKUP(J2,Res,28,0)</f>
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="AC2" s="28">
         <f t="shared" ref="AC2:AC33" si="18">VLOOKUP(I2,Res,31,0)*AD2+AE2</f>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="AF2">
         <f>VLOOKUP(AB2,verftab,2,1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG2" s="162">
         <v>0</v>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="AB3" s="27">
         <f t="shared" si="17"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC3" s="28">
         <f t="shared" si="18"/>
@@ -3083,8 +3083,8 @@
         <v>229.9</v>
       </c>
       <c r="AF3">
-        <f t="shared" ref="AF2:AF33" si="21">VLOOKUP(AB3,verftab,2,1)</f>
-        <v>3</v>
+        <f t="shared" ref="AF3:AF33" si="21">VLOOKUP(AB3,verftab,2,1)</f>
+        <v>4</v>
       </c>
       <c r="AG3" s="162">
         <v>0</v>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="AB4" s="27">
         <f t="shared" si="17"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC4" s="28">
         <f t="shared" si="18"/>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="AF4">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG4" s="162">
         <v>0</v>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="AB5" s="27">
         <f t="shared" si="17"/>
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AC5" s="28">
         <f t="shared" si="18"/>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="AF5">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG5" s="162">
         <v>0</v>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="AB6" s="27">
         <f t="shared" si="17"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC6" s="28">
         <f t="shared" si="18"/>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AF6">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG6" s="162">
         <v>0</v>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AB7" s="27">
         <f t="shared" si="17"/>
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AC7" s="28">
         <f t="shared" si="18"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="AF7">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG7" s="162">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="AB8" s="27">
         <f t="shared" si="17"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC8" s="28">
         <f t="shared" si="18"/>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="AF8">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG8" s="162">
         <v>0</v>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="AB9" s="27">
         <f t="shared" si="17"/>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="AC9" s="28">
         <f t="shared" si="18"/>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="AB10" s="27">
         <f t="shared" si="17"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC10" s="28">
         <f t="shared" si="18"/>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="AF10">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG10" s="162">
         <v>0</v>
@@ -4052,7 +4052,7 @@
       </c>
       <c r="AB11" s="27">
         <f t="shared" si="17"/>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AC11" s="28">
         <f t="shared" si="18"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="AF11">
         <f t="shared" si="21"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG11" s="162">
         <v>0</v>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="AB12" s="27">
         <f t="shared" si="17"/>
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="AC12" s="28">
         <f t="shared" si="18"/>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="AF12">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG12" s="162">
         <v>0</v>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="AB13" s="27">
         <f t="shared" si="17"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="AC13" s="28">
         <f t="shared" si="18"/>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="AB14" s="27">
         <f t="shared" si="17"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC14" s="28">
         <f t="shared" si="18"/>
@@ -4437,7 +4437,7 @@
       </c>
       <c r="AF14">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG14" s="162">
         <v>0</v>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="AB15" s="27">
         <f t="shared" si="17"/>
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="AC15" s="28">
         <f t="shared" si="18"/>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="AB16" s="27">
         <f t="shared" si="17"/>
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="AC16" s="28">
         <f t="shared" si="18"/>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="AF16">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG16" s="162">
         <v>0</v>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="AB17" s="27">
         <f t="shared" si="17"/>
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="AC17" s="28">
         <f t="shared" si="18"/>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="AF17">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG17" s="162">
         <v>0</v>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="AB18" s="27">
         <f t="shared" si="17"/>
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="AC18" s="28">
         <f t="shared" si="18"/>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="AF18">
         <f t="shared" si="21"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG18" s="162">
         <v>0</v>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="AB19" s="27">
         <f t="shared" si="17"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="AC19" s="28">
         <f t="shared" si="18"/>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="AB20" s="27">
         <f t="shared" si="17"/>
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="AC20" s="28">
         <f t="shared" si="18"/>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="AF20">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG20" s="162">
         <v>0</v>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="AB21" s="27">
         <f t="shared" si="17"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC21" s="28">
         <f t="shared" si="18"/>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="AF21">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG21" s="162">
         <v>0</v>
@@ -5405,7 +5405,7 @@
       </c>
       <c r="AB22" s="27">
         <f t="shared" si="17"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC22" s="28">
         <f t="shared" si="18"/>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="AF22">
         <f t="shared" si="21"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG22" s="162">
         <v>0</v>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="AB23" s="27">
         <f t="shared" si="17"/>
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AC23" s="28">
         <f t="shared" si="18"/>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="AF23">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG23" s="162">
         <v>0</v>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="AB24" s="27">
         <f t="shared" si="17"/>
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="AC24" s="28">
         <f t="shared" si="18"/>
@@ -5667,7 +5667,7 @@
       </c>
       <c r="AF24">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG24" s="162">
         <v>0</v>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="AB25" s="27">
         <f t="shared" si="17"/>
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="AC25" s="28">
         <f t="shared" si="18"/>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="AF25">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG25" s="162">
         <v>0</v>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="AB26" s="27">
         <f t="shared" si="17"/>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AC26" s="28">
         <f t="shared" si="18"/>
@@ -5913,7 +5913,7 @@
       </c>
       <c r="AF26">
         <f t="shared" si="21"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG26" s="162">
         <v>0</v>
@@ -6020,7 +6020,7 @@
       </c>
       <c r="AB27" s="27">
         <f t="shared" si="17"/>
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="AC27" s="28">
         <f t="shared" si="18"/>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="AF27">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG27" s="162">
         <v>0</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="AB28" s="27">
         <f t="shared" si="17"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC28" s="28">
         <f t="shared" si="18"/>
@@ -6159,7 +6159,7 @@
       </c>
       <c r="AF28">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG28" s="162">
         <v>0</v>
@@ -6266,7 +6266,7 @@
       </c>
       <c r="AB29" s="27">
         <f t="shared" si="17"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC29" s="28">
         <f t="shared" si="18"/>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="AF29">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG29" s="162">
         <v>0</v>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="AB30" s="27">
         <f t="shared" si="17"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC30" s="28">
         <f t="shared" si="18"/>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="AF30">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG30" s="162">
         <v>0</v>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="AB31" s="27">
         <f t="shared" si="17"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC31" s="28">
         <f t="shared" si="18"/>
@@ -6528,7 +6528,7 @@
       </c>
       <c r="AF31">
         <f t="shared" si="21"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG31" s="162">
         <v>0</v>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="AB32" s="27">
         <f t="shared" si="17"/>
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="AC32" s="28">
         <f t="shared" si="18"/>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="AF32">
         <f t="shared" si="21"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG32" s="162">
         <v>0</v>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="AB33" s="27">
         <f t="shared" si="17"/>
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="AC33" s="28">
         <f t="shared" si="18"/>
@@ -6774,7 +6774,7 @@
       </c>
       <c r="AF33">
         <f t="shared" si="21"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG33" s="162">
         <v>0</v>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="AB34" s="27">
         <f t="shared" ref="AB34:AB65" si="39">VLOOKUP(B34,Res,28,0)+VLOOKUP(C34,Res,28,0)+VLOOKUP(D34,Res,28,0)+VLOOKUP(E34,Res,28,0)+VLOOKUP(F34,Res,28,0)+VLOOKUP(G34,Res,28,0)+VLOOKUP(I34,Res,28,0)+VLOOKUP(J34,Res,28,0)</f>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC34" s="28">
         <f t="shared" ref="AC34:AC65" si="40">VLOOKUP(I34,Res,31,0)*AD34+AE34</f>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="AF34">
         <f t="shared" ref="AF34:AF65" si="43">VLOOKUP(AB34,verftab,2,1)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG34" s="162">
         <v>0</v>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="AB35" s="27">
         <f t="shared" si="39"/>
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="AC35" s="28">
         <f t="shared" si="40"/>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="AF35">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG35" s="162">
         <v>0</v>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="AB36" s="27">
         <f t="shared" si="39"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC36" s="28">
         <f t="shared" si="40"/>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="AF36">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG36" s="162">
         <v>0</v>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="AB37" s="27">
         <f t="shared" si="39"/>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="AC37" s="28">
         <f t="shared" si="40"/>
@@ -7266,7 +7266,7 @@
       </c>
       <c r="AF37">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG37" s="162">
         <v>0</v>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="AB38" s="27">
         <f t="shared" si="39"/>
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="AC38" s="28">
         <f t="shared" si="40"/>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="AF38">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG38" s="162">
         <v>0</v>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="AB39" s="27">
         <f t="shared" si="39"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC39" s="28">
         <f t="shared" si="40"/>
@@ -7512,7 +7512,7 @@
       </c>
       <c r="AF39">
         <f t="shared" si="43"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG39" s="162">
         <v>0</v>
@@ -7619,7 +7619,7 @@
       </c>
       <c r="AB40" s="27">
         <f t="shared" si="39"/>
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="AC40" s="28">
         <f t="shared" si="40"/>
@@ -7635,7 +7635,7 @@
       </c>
       <c r="AF40">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG40" s="162">
         <v>0</v>
@@ -7742,7 +7742,7 @@
       </c>
       <c r="AB41" s="27">
         <f t="shared" si="39"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC41" s="28">
         <f t="shared" si="40"/>
@@ -7758,7 +7758,7 @@
       </c>
       <c r="AF41">
         <f t="shared" si="43"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG41" s="162">
         <v>0</v>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="AB42" s="27">
         <f t="shared" si="39"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC42" s="28">
         <f t="shared" si="40"/>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="AF42">
         <f t="shared" si="43"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG42" s="162">
         <v>0</v>
@@ -7988,7 +7988,7 @@
       </c>
       <c r="AB43" s="27">
         <f t="shared" si="39"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC43" s="28">
         <f t="shared" si="40"/>
@@ -8004,7 +8004,7 @@
       </c>
       <c r="AF43">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG43" s="162">
         <v>0</v>
@@ -8111,7 +8111,7 @@
       </c>
       <c r="AB44" s="27">
         <f t="shared" si="39"/>
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="AC44" s="28">
         <f t="shared" si="40"/>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="AF44">
         <f t="shared" si="43"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG44" s="162">
         <v>0</v>
@@ -8234,7 +8234,7 @@
       </c>
       <c r="AB45" s="27">
         <f t="shared" si="39"/>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="AC45" s="28">
         <f t="shared" si="40"/>
@@ -8250,7 +8250,7 @@
       </c>
       <c r="AF45">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG45" s="162">
         <v>0</v>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="AB46" s="27">
         <f t="shared" si="39"/>
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="AC46" s="28">
         <f t="shared" si="40"/>
@@ -8373,7 +8373,7 @@
       </c>
       <c r="AF46">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG46" s="162">
         <v>0</v>
@@ -8480,7 +8480,7 @@
       </c>
       <c r="AB47" s="27">
         <f t="shared" si="39"/>
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="AC47" s="28">
         <f t="shared" si="40"/>
@@ -8496,7 +8496,7 @@
       </c>
       <c r="AF47">
         <f t="shared" si="43"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG47" s="162">
         <v>0</v>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="AB48" s="27">
         <f t="shared" si="39"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC48" s="28">
         <f t="shared" si="40"/>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="AF48">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG48" s="162">
         <v>0</v>
@@ -8726,7 +8726,7 @@
       </c>
       <c r="AB49" s="27">
         <f t="shared" si="39"/>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="AC49" s="28">
         <f t="shared" si="40"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="AF49">
         <f t="shared" si="43"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG49" s="162">
         <v>0</v>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="AB50" s="27">
         <f t="shared" si="39"/>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="AC50" s="28">
         <f t="shared" si="40"/>
@@ -8865,7 +8865,7 @@
       </c>
       <c r="AF50">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG50" s="162">
         <v>0</v>
@@ -8972,7 +8972,7 @@
       </c>
       <c r="AB51" s="27">
         <f t="shared" si="39"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC51" s="28">
         <f t="shared" si="40"/>
@@ -8988,7 +8988,7 @@
       </c>
       <c r="AF51">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG51" s="162">
         <v>0</v>
@@ -9095,7 +9095,7 @@
       </c>
       <c r="AB52" s="27">
         <f t="shared" si="39"/>
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AC52" s="28">
         <f t="shared" si="40"/>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="AF52">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG52" s="162">
         <v>0</v>
@@ -9218,7 +9218,7 @@
       </c>
       <c r="AB53" s="27">
         <f t="shared" si="39"/>
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="AC53" s="28">
         <f t="shared" si="40"/>
@@ -9234,7 +9234,7 @@
       </c>
       <c r="AF53">
         <f t="shared" si="43"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG53" s="162">
         <v>0</v>
@@ -9341,7 +9341,7 @@
       </c>
       <c r="AB54" s="27">
         <f t="shared" si="39"/>
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="AC54" s="28">
         <f t="shared" si="40"/>
@@ -9357,7 +9357,7 @@
       </c>
       <c r="AF54">
         <f t="shared" si="43"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG54" s="162">
         <v>0</v>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="AB55" s="27">
         <f t="shared" si="39"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC55" s="28">
         <f t="shared" si="40"/>
@@ -9480,7 +9480,7 @@
       </c>
       <c r="AF55">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG55" s="162">
         <v>0</v>
@@ -9587,7 +9587,7 @@
       </c>
       <c r="AB56" s="27">
         <f t="shared" si="39"/>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="AC56" s="28">
         <f t="shared" si="40"/>
@@ -9603,7 +9603,7 @@
       </c>
       <c r="AF56">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG56" s="162">
         <v>0</v>
@@ -9710,7 +9710,7 @@
       </c>
       <c r="AB57" s="27">
         <f t="shared" si="39"/>
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="AC57" s="28">
         <f t="shared" si="40"/>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="AF57">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG57" s="162">
         <v>0</v>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="AB58" s="27">
         <f t="shared" si="39"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC58" s="28">
         <f t="shared" si="40"/>
@@ -9849,7 +9849,7 @@
       </c>
       <c r="AF58">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG58" s="162">
         <v>0</v>
@@ -9956,7 +9956,7 @@
       </c>
       <c r="AB59" s="27">
         <f t="shared" si="39"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC59" s="28">
         <f t="shared" si="40"/>
@@ -9972,7 +9972,7 @@
       </c>
       <c r="AF59">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG59" s="162">
         <v>0</v>
@@ -10079,7 +10079,7 @@
       </c>
       <c r="AB60" s="27">
         <f t="shared" si="39"/>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AC60" s="28">
         <f t="shared" si="40"/>
@@ -10095,7 +10095,7 @@
       </c>
       <c r="AF60">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG60" s="162">
         <v>0</v>
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AB61" s="27">
         <f t="shared" si="39"/>
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="AC61" s="28">
         <f t="shared" si="40"/>
@@ -10218,7 +10218,7 @@
       </c>
       <c r="AF61">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG61" s="162">
         <v>0</v>
@@ -10325,7 +10325,7 @@
       </c>
       <c r="AB62" s="27">
         <f t="shared" si="39"/>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AC62" s="28">
         <f t="shared" si="40"/>
@@ -10341,7 +10341,7 @@
       </c>
       <c r="AF62">
         <f t="shared" si="43"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG62" s="162">
         <v>0</v>
@@ -10448,7 +10448,7 @@
       </c>
       <c r="AB63" s="27">
         <f t="shared" si="39"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC63" s="28">
         <f t="shared" si="40"/>
@@ -10464,7 +10464,7 @@
       </c>
       <c r="AF63">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG63" s="162">
         <v>0</v>
@@ -10571,7 +10571,7 @@
       </c>
       <c r="AB64" s="27">
         <f t="shared" si="39"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC64" s="28">
         <f t="shared" si="40"/>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="AF64">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG64" s="162">
         <v>0</v>
@@ -10694,7 +10694,7 @@
       </c>
       <c r="AB65" s="27">
         <f t="shared" si="39"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC65" s="28">
         <f t="shared" si="40"/>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="AF65">
         <f t="shared" si="43"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG65" s="162">
         <v>0</v>
@@ -10817,7 +10817,7 @@
       </c>
       <c r="AB66" s="27">
         <f t="shared" ref="AB66:AB87" si="61">VLOOKUP(B66,Res,28,0)+VLOOKUP(C66,Res,28,0)+VLOOKUP(D66,Res,28,0)+VLOOKUP(E66,Res,28,0)+VLOOKUP(F66,Res,28,0)+VLOOKUP(G66,Res,28,0)+VLOOKUP(I66,Res,28,0)+VLOOKUP(J66,Res,28,0)</f>
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="AC66" s="28">
         <f t="shared" ref="AC66:AC87" si="62">VLOOKUP(I66,Res,31,0)*AD66+AE66</f>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="AF66">
         <f t="shared" ref="AF66:AF87" si="65">VLOOKUP(AB66,verftab,2,1)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG66" s="162">
         <v>0</v>
@@ -10940,7 +10940,7 @@
       </c>
       <c r="AB67" s="27">
         <f t="shared" si="61"/>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AC67" s="28">
         <f t="shared" si="62"/>
@@ -10956,7 +10956,7 @@
       </c>
       <c r="AF67">
         <f t="shared" si="65"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG67" s="162">
         <v>0</v>
@@ -11063,7 +11063,7 @@
       </c>
       <c r="AB68" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC68" s="28">
         <f t="shared" si="62"/>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="AF68">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG68" s="162">
         <v>0</v>
@@ -11186,7 +11186,7 @@
       </c>
       <c r="AB69" s="27">
         <f t="shared" si="61"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC69" s="28">
         <f t="shared" si="62"/>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="AF69">
         <f t="shared" si="65"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG69" s="162">
         <v>0</v>
@@ -11309,7 +11309,7 @@
       </c>
       <c r="AB70" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC70" s="28">
         <f t="shared" si="62"/>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="AF70">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG70" s="162">
         <v>0</v>
@@ -11432,7 +11432,7 @@
       </c>
       <c r="AB71" s="27">
         <f t="shared" si="61"/>
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="AC71" s="28">
         <f t="shared" si="62"/>
@@ -11448,7 +11448,7 @@
       </c>
       <c r="AF71">
         <f t="shared" si="65"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG71" s="162">
         <v>0</v>
@@ -11555,7 +11555,7 @@
       </c>
       <c r="AB72" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC72" s="28">
         <f t="shared" si="62"/>
@@ -11571,7 +11571,7 @@
       </c>
       <c r="AF72">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG72" s="162">
         <v>0</v>
@@ -11678,7 +11678,7 @@
       </c>
       <c r="AB73" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC73" s="28">
         <f t="shared" si="62"/>
@@ -11694,7 +11694,7 @@
       </c>
       <c r="AF73">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG73" s="162">
         <v>0</v>
@@ -11801,7 +11801,7 @@
       </c>
       <c r="AB74" s="27">
         <f t="shared" si="61"/>
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AC74" s="28">
         <f t="shared" si="62"/>
@@ -11817,7 +11817,7 @@
       </c>
       <c r="AF74">
         <f t="shared" si="65"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG74" s="162">
         <v>0</v>
@@ -11924,7 +11924,7 @@
       </c>
       <c r="AB75" s="27">
         <f t="shared" si="61"/>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="AC75" s="28">
         <f t="shared" si="62"/>
@@ -11940,7 +11940,7 @@
       </c>
       <c r="AF75">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG75" s="162">
         <v>0</v>
@@ -12047,7 +12047,7 @@
       </c>
       <c r="AB76" s="27">
         <f t="shared" si="61"/>
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AC76" s="28">
         <f t="shared" si="62"/>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="AF76">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG76" s="162">
         <v>0</v>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="AB77" s="27">
         <f t="shared" si="61"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC77" s="28">
         <f t="shared" si="62"/>
@@ -12186,7 +12186,7 @@
       </c>
       <c r="AF77">
         <f t="shared" si="65"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG77" s="162">
         <v>0</v>
@@ -12293,7 +12293,7 @@
       </c>
       <c r="AB78" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC78" s="28">
         <f t="shared" si="62"/>
@@ -12309,7 +12309,7 @@
       </c>
       <c r="AF78">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG78" s="162">
         <v>0</v>
@@ -12416,7 +12416,7 @@
       </c>
       <c r="AB79" s="27">
         <f t="shared" si="61"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="AC79" s="28">
         <f t="shared" si="62"/>
@@ -12539,7 +12539,7 @@
       </c>
       <c r="AB80" s="27">
         <f t="shared" si="61"/>
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="AC80" s="28">
         <f t="shared" si="62"/>
@@ -12555,7 +12555,7 @@
       </c>
       <c r="AF80">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG80" s="162">
         <v>0</v>
@@ -12662,7 +12662,7 @@
       </c>
       <c r="AB81" s="27">
         <f t="shared" si="61"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="AC81" s="28">
         <f t="shared" si="62"/>
@@ -12785,7 +12785,7 @@
       </c>
       <c r="AB82" s="27">
         <f t="shared" si="61"/>
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="AC82" s="28">
         <f t="shared" si="62"/>
@@ -12801,7 +12801,7 @@
       </c>
       <c r="AF82">
         <f t="shared" si="65"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG82" s="162">
         <v>0</v>
@@ -12908,7 +12908,7 @@
       </c>
       <c r="AB83" s="27">
         <f t="shared" si="61"/>
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="AC83" s="28">
         <f t="shared" si="62"/>
@@ -12924,7 +12924,7 @@
       </c>
       <c r="AF83">
         <f t="shared" si="65"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG83" s="162">
         <v>0</v>
@@ -13031,7 +13031,7 @@
       </c>
       <c r="AB84" s="27">
         <f t="shared" si="61"/>
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="AC84" s="28">
         <f t="shared" si="62"/>
@@ -13047,7 +13047,7 @@
       </c>
       <c r="AF84">
         <f t="shared" si="65"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG84" s="162">
         <v>0</v>
@@ -13154,7 +13154,7 @@
       </c>
       <c r="AB85" s="27">
         <f t="shared" si="61"/>
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="AC85" s="28">
         <f t="shared" si="62"/>
@@ -13170,7 +13170,7 @@
       </c>
       <c r="AF85">
         <f t="shared" si="65"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG85" s="162">
         <v>0</v>
@@ -13277,7 +13277,7 @@
       </c>
       <c r="AB86" s="27">
         <f t="shared" si="61"/>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="AC86" s="28">
         <f t="shared" si="62"/>
@@ -13400,7 +13400,7 @@
       </c>
       <c r="AB87" s="27">
         <f t="shared" si="61"/>
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="AC87" s="28">
         <f t="shared" si="62"/>
@@ -13416,7 +13416,7 @@
       </c>
       <c r="AF87">
         <f t="shared" si="65"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG87" s="162">
         <v>0</v>
@@ -18406,7 +18406,7 @@
         <v>5</v>
       </c>
       <c r="AB32" s="94">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="AC32" s="94"/>
       <c r="AD32" s="96"/>
@@ -18465,7 +18465,7 @@
         <v>-3</v>
       </c>
       <c r="AB33" s="94">
-        <v>-30</v>
+        <v>3</v>
       </c>
       <c r="AC33" s="94"/>
       <c r="AD33" s="94"/>
@@ -18509,7 +18509,9 @@
       <c r="Y34" s="94"/>
       <c r="Z34" s="94"/>
       <c r="AA34" s="94"/>
-      <c r="AB34" s="94"/>
+      <c r="AB34" s="94">
+        <v>0</v>
+      </c>
       <c r="AC34" s="94"/>
       <c r="AD34" s="94"/>
       <c r="AE34" s="97">
@@ -18567,7 +18569,7 @@
         <v>3</v>
       </c>
       <c r="AB35" s="94">
-        <v>30</v>
+        <v>-1</v>
       </c>
       <c r="AC35" s="94"/>
       <c r="AD35" s="96">
@@ -18632,7 +18634,7 @@
         <v>-2</v>
       </c>
       <c r="AB36" s="94">
-        <v>-20</v>
+        <v>2</v>
       </c>
       <c r="AC36" s="94"/>
       <c r="AD36" s="94"/>
@@ -18691,7 +18693,7 @@
         <v>2</v>
       </c>
       <c r="AB37" s="94">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="AC37" s="94"/>
       <c r="AD37" s="96">
@@ -18756,7 +18758,7 @@
         <v>-1</v>
       </c>
       <c r="AB38" s="94">
-        <v>-10</v>
+        <v>1</v>
       </c>
       <c r="AC38" s="94"/>
       <c r="AD38" s="94"/>
@@ -19048,7 +19050,7 @@
       <c r="Z44" s="117"/>
       <c r="AA44" s="117"/>
       <c r="AB44" s="117">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AC44" s="117"/>
       <c r="AD44" s="119">
@@ -19105,7 +19107,7 @@
       <c r="Z45" s="117"/>
       <c r="AA45" s="117"/>
       <c r="AB45" s="117">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="AC45" s="117"/>
       <c r="AD45" s="119">
@@ -19149,7 +19151,9 @@
       <c r="Y46" s="117"/>
       <c r="Z46" s="117"/>
       <c r="AA46" s="117"/>
-      <c r="AB46" s="117"/>
+      <c r="AB46" s="117">
+        <v>0</v>
+      </c>
       <c r="AC46" s="117"/>
       <c r="AD46" s="119"/>
       <c r="AE46" s="117"/>

</xml_diff>

<commit_message>
Update firearm and game value spreadsheets
</commit_message>
<xml_diff>
--- a/NN_Feuerwaffen_1.1.xlsx
+++ b/NN_Feuerwaffen_1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Das Western Rollenspiel\LLM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09394C19-92EE-4C47-82E4-B1B3CD670A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848433D3-7E6E-408B-BBAC-E26BFA4D68C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23655" yWindow="525" windowWidth="26010" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3555" yWindow="135" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Waffen" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="384">
   <si>
     <t>Name</t>
   </si>
@@ -1201,6 +1201,15 @@
   </si>
   <si>
     <t>Ini</t>
+  </si>
+  <si>
+    <t>16mm</t>
+  </si>
+  <si>
+    <t>17mm</t>
+  </si>
+  <si>
+    <t>harpune</t>
   </si>
 </sst>
 </file>
@@ -1919,7 +1928,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2365,6 +2374,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -13473,7 +13486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AMK35"/>
+  <dimension ref="A1:AMK40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="162" customWidth="1"/>
@@ -14503,7 +14516,7 @@
         <v>721.50666666666677</v>
       </c>
     </row>
-    <row r="29" spans="1:10" s="55" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" s="55" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="48" t="s">
         <v>54</v>
       </c>
@@ -14539,7 +14552,7 @@
       </c>
       <c r="J29" s="54"/>
     </row>
-    <row r="30" spans="1:10" s="67" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" s="172" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="60" t="s">
         <v>174</v>
       </c>
@@ -14547,103 +14560,105 @@
         <v>175</v>
       </c>
       <c r="C30" s="62">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D30" s="63">
         <f>'Ressourcen-Munition'!D51</f>
-        <v>0.78139999999999998</v>
+        <v>0.40360320000000005</v>
       </c>
       <c r="E30" s="64">
         <f>'Ressourcen-Munition'!E51</f>
-        <v>7.8140000000000001</v>
+        <v>4.0360320000000005</v>
       </c>
       <c r="F30" s="65">
         <f>'Ressourcen-Munition'!F51</f>
-        <v>39.07</v>
+        <v>20.180160000000001</v>
       </c>
       <c r="G30" s="65">
         <f>'Ressourcen-Munition'!G51</f>
-        <v>78.14</v>
+        <v>40.360320000000002</v>
       </c>
       <c r="H30" s="65">
         <f>'Ressourcen-Munition'!H51</f>
-        <v>390.7</v>
+        <v>201.80160000000004</v>
       </c>
       <c r="I30" s="65">
         <f>'Ressourcen-Munition'!I51</f>
-        <v>781.4</v>
-      </c>
-      <c r="J30" s="66"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="162" t="s">
+        <v>403.60320000000007</v>
+      </c>
+      <c r="J30" s="171"/>
+    </row>
+    <row r="31" spans="1:10" s="172" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="60" t="s">
         <v>174</v>
       </c>
-      <c r="B31" s="71" t="s">
+      <c r="B31" s="70" t="s">
         <v>175</v>
       </c>
-      <c r="C31" s="45">
-        <v>8</v>
-      </c>
-      <c r="D31" s="46">
+      <c r="C31" s="62">
+        <v>6</v>
+      </c>
+      <c r="D31" s="63">
         <f>'Ressourcen-Munition'!D52</f>
-        <v>0.82515840000000007</v>
-      </c>
-      <c r="E31" s="47">
+        <v>0.44510400000000006</v>
+      </c>
+      <c r="E31" s="64">
         <f>'Ressourcen-Munition'!E52</f>
-        <v>8.2515840000000011</v>
-      </c>
-      <c r="F31" s="57">
+        <v>4.4510400000000008</v>
+      </c>
+      <c r="F31" s="65">
         <f>'Ressourcen-Munition'!F52</f>
-        <v>41.257920000000006</v>
-      </c>
-      <c r="G31" s="57">
+        <v>22.255200000000002</v>
+      </c>
+      <c r="G31" s="65">
         <f>'Ressourcen-Munition'!G52</f>
-        <v>82.515840000000011</v>
-      </c>
-      <c r="H31" s="57">
+        <v>44.510400000000004</v>
+      </c>
+      <c r="H31" s="65">
         <f>'Ressourcen-Munition'!H52</f>
-        <v>412.57920000000001</v>
-      </c>
-      <c r="I31" s="57">
+        <v>222.55200000000002</v>
+      </c>
+      <c r="I31" s="65">
         <f>'Ressourcen-Munition'!I52</f>
-        <v>825.15840000000003</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="162" t="s">
+        <v>445.10400000000004</v>
+      </c>
+      <c r="J31" s="171"/>
+    </row>
+    <row r="32" spans="1:10" s="67" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="60" t="s">
         <v>174</v>
       </c>
-      <c r="B32" s="71" t="s">
+      <c r="B32" s="70" t="s">
         <v>175</v>
       </c>
-      <c r="C32" s="45">
-        <v>9</v>
-      </c>
-      <c r="D32" s="46">
+      <c r="C32" s="62">
+        <v>7</v>
+      </c>
+      <c r="D32" s="63">
         <f>'Ressourcen-Munition'!D53</f>
-        <v>0.86891680000000004</v>
-      </c>
-      <c r="E32" s="47">
+        <v>0.71878400000000009</v>
+      </c>
+      <c r="E32" s="64">
         <f>'Ressourcen-Munition'!E53</f>
-        <v>8.6891680000000004</v>
-      </c>
-      <c r="F32" s="57">
+        <v>7.1878400000000013</v>
+      </c>
+      <c r="F32" s="65">
         <f>'Ressourcen-Munition'!F53</f>
-        <v>43.445840000000004</v>
-      </c>
-      <c r="G32" s="57">
+        <v>35.939200000000007</v>
+      </c>
+      <c r="G32" s="65">
         <f>'Ressourcen-Munition'!G53</f>
-        <v>86.891680000000008</v>
-      </c>
-      <c r="H32" s="57">
+        <v>71.878400000000013</v>
+      </c>
+      <c r="H32" s="65">
         <f>'Ressourcen-Munition'!H53</f>
-        <v>434.45840000000004</v>
-      </c>
-      <c r="I32" s="57">
+        <v>359.39200000000005</v>
+      </c>
+      <c r="I32" s="65">
         <f>'Ressourcen-Munition'!I53</f>
-        <v>868.91680000000008</v>
-      </c>
+        <v>718.78400000000011</v>
+      </c>
+      <c r="J32" s="66"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="162" t="s">
@@ -14653,31 +14668,31 @@
         <v>175</v>
       </c>
       <c r="C33" s="45">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D33" s="46">
         <f>'Ressourcen-Munition'!D54</f>
-        <v>0.91267519999999991</v>
+        <v>0.82515840000000007</v>
       </c>
       <c r="E33" s="47">
         <f>'Ressourcen-Munition'!E54</f>
-        <v>9.1267519999999998</v>
+        <v>8.2515840000000011</v>
       </c>
       <c r="F33" s="57">
         <f>'Ressourcen-Munition'!F54</f>
-        <v>45.633759999999995</v>
+        <v>41.257920000000006</v>
       </c>
       <c r="G33" s="57">
         <f>'Ressourcen-Munition'!G54</f>
-        <v>91.26751999999999</v>
+        <v>82.515840000000011</v>
       </c>
       <c r="H33" s="57">
         <f>'Ressourcen-Munition'!H54</f>
-        <v>456.33759999999995</v>
+        <v>412.57920000000001</v>
       </c>
       <c r="I33" s="57">
         <f>'Ressourcen-Munition'!I54</f>
-        <v>912.6751999999999</v>
+        <v>825.15840000000003</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -14688,31 +14703,31 @@
         <v>175</v>
       </c>
       <c r="C34" s="45">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D34" s="46">
         <f>'Ressourcen-Munition'!D55</f>
-        <v>0.95643359999999999</v>
+        <v>0.86891680000000004</v>
       </c>
       <c r="E34" s="47">
         <f>'Ressourcen-Munition'!E55</f>
-        <v>9.5643360000000008</v>
+        <v>8.6891680000000004</v>
       </c>
       <c r="F34" s="57">
         <f>'Ressourcen-Munition'!F55</f>
-        <v>47.821680000000001</v>
+        <v>43.445840000000004</v>
       </c>
       <c r="G34" s="57">
         <f>'Ressourcen-Munition'!G55</f>
-        <v>95.643360000000001</v>
+        <v>86.891680000000008</v>
       </c>
       <c r="H34" s="57">
         <f>'Ressourcen-Munition'!H55</f>
-        <v>478.21679999999998</v>
+        <v>434.45840000000004</v>
       </c>
       <c r="I34" s="57">
         <f>'Ressourcen-Munition'!I55</f>
-        <v>956.43359999999996</v>
+        <v>868.91680000000008</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -14723,32 +14738,135 @@
         <v>175</v>
       </c>
       <c r="C35" s="45">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D35" s="46">
         <f>'Ressourcen-Munition'!D56</f>
-        <v>1.000192</v>
+        <v>0.91267519999999991</v>
       </c>
       <c r="E35" s="47">
         <f>'Ressourcen-Munition'!E56</f>
-        <v>10.00192</v>
+        <v>9.1267519999999998</v>
       </c>
       <c r="F35" s="57">
         <f>'Ressourcen-Munition'!F56</f>
-        <v>50.009599999999999</v>
+        <v>45.633759999999995</v>
       </c>
       <c r="G35" s="57">
         <f>'Ressourcen-Munition'!G56</f>
-        <v>100.0192</v>
+        <v>91.26751999999999</v>
       </c>
       <c r="H35" s="57">
         <f>'Ressourcen-Munition'!H56</f>
-        <v>500.096</v>
+        <v>456.33759999999995</v>
       </c>
       <c r="I35" s="57">
         <f>'Ressourcen-Munition'!I56</f>
+        <v>912.6751999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="162" t="s">
+        <v>174</v>
+      </c>
+      <c r="B36" s="71" t="s">
+        <v>175</v>
+      </c>
+      <c r="C36" s="45">
+        <v>11</v>
+      </c>
+      <c r="D36" s="46">
+        <f>'Ressourcen-Munition'!D57</f>
+        <v>0.95643359999999999</v>
+      </c>
+      <c r="E36" s="47">
+        <f>'Ressourcen-Munition'!E57</f>
+        <v>9.5643360000000008</v>
+      </c>
+      <c r="F36" s="57">
+        <f>'Ressourcen-Munition'!F57</f>
+        <v>47.821680000000001</v>
+      </c>
+      <c r="G36" s="57">
+        <f>'Ressourcen-Munition'!G57</f>
+        <v>95.643360000000001</v>
+      </c>
+      <c r="H36" s="57">
+        <f>'Ressourcen-Munition'!H57</f>
+        <v>478.21679999999998</v>
+      </c>
+      <c r="I36" s="57">
+        <f>'Ressourcen-Munition'!I57</f>
+        <v>956.43359999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="162" t="s">
+        <v>174</v>
+      </c>
+      <c r="B37" s="71" t="s">
+        <v>175</v>
+      </c>
+      <c r="C37" s="45">
+        <v>12</v>
+      </c>
+      <c r="D37" s="46">
+        <f>'Ressourcen-Munition'!D58</f>
+        <v>1.000192</v>
+      </c>
+      <c r="E37" s="47">
+        <f>'Ressourcen-Munition'!E58</f>
+        <v>10.00192</v>
+      </c>
+      <c r="F37" s="57">
+        <f>'Ressourcen-Munition'!F58</f>
+        <v>50.009599999999999</v>
+      </c>
+      <c r="G37" s="57">
+        <f>'Ressourcen-Munition'!G58</f>
+        <v>100.0192</v>
+      </c>
+      <c r="H37" s="57">
+        <f>'Ressourcen-Munition'!H58</f>
+        <v>500.096</v>
+      </c>
+      <c r="I37" s="57">
+        <f>'Ressourcen-Munition'!I58</f>
         <v>1000.192</v>
       </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="162" t="s">
+        <v>108</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="D38" s="46">
+        <f>'Ressourcen-Munition'!D59</f>
+        <v>6.8838400000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="162" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="D39" s="46">
+        <f>'Ressourcen-Munition'!D60</f>
+        <v>6.8838400000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -19599,7 +19717,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AMK56"/>
+  <dimension ref="A1:AMK60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1025" width="11.42578125" style="59" customWidth="1"/>
@@ -19696,6 +19814,12 @@
         <f>C5*0.8</f>
         <v>12</v>
       </c>
+      <c r="E5" s="59" t="s">
+        <v>109</v>
+      </c>
+      <c r="F5" s="152">
+        <v>3</v>
+      </c>
       <c r="L5" s="130"/>
       <c r="N5" s="131"/>
     </row>
@@ -19970,7 +20094,7 @@
       </c>
       <c r="O16" s="166"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -19989,19 +20113,19 @@
         <v>2.4E-2</v>
       </c>
       <c r="G17" s="154">
-        <f>(B17*G11)</f>
+        <f>(B17*$G$11)</f>
         <v>0.34</v>
       </c>
       <c r="H17" s="154">
-        <f>(C17*H11)</f>
+        <f>(C17*$H$11)</f>
         <v>3.8400000000000004E-2</v>
       </c>
       <c r="I17" s="154">
-        <f>(D17*I11)</f>
+        <f>(D17*$I$11)</f>
         <v>0</v>
       </c>
       <c r="J17" s="154">
-        <f>(E17*J11)</f>
+        <f>(E17*$J$11)</f>
         <v>0.38400000000000001</v>
       </c>
       <c r="K17" s="158">
@@ -20012,7 +20136,7 @@
         <v>2000</v>
       </c>
       <c r="M17" s="159">
-        <f>F6/L17</f>
+        <f>$F$6/L17</f>
         <v>1.9E-2</v>
       </c>
       <c r="N17" s="163">
@@ -20021,6 +20145,56 @@
       </c>
       <c r="O17" s="164"/>
     </row>
+    <row r="18" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="59" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="152">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="C18" s="152">
+        <v>0.05</v>
+      </c>
+      <c r="E18" s="59">
+        <v>0.15</v>
+      </c>
+      <c r="F18" s="157">
+        <f>B18+C18+D18+E18</f>
+        <v>0.215</v>
+      </c>
+      <c r="G18" s="154">
+        <f>(B18*$G$11)</f>
+        <v>1.02</v>
+      </c>
+      <c r="H18" s="154">
+        <f>(C18*$H$11)</f>
+        <v>0.48000000000000009</v>
+      </c>
+      <c r="I18" s="154">
+        <f>(D18*$I$11)</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="154">
+        <f>(E18*$J$11)</f>
+        <v>3.84</v>
+      </c>
+      <c r="K18" s="158">
+        <f>G18+H18+I18+J18</f>
+        <v>5.34</v>
+      </c>
+      <c r="L18" s="150">
+        <v>1000</v>
+      </c>
+      <c r="M18" s="159">
+        <f>$F$6/L18</f>
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="N18" s="163">
+        <f>M18+K18</f>
+        <v>5.3780000000000001</v>
+      </c>
+      <c r="O18" s="164"/>
+    </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>0</v>
@@ -20062,23 +20236,23 @@
         <v>0.36691200000000002</v>
       </c>
       <c r="E23" s="131">
-        <f t="shared" ref="E23:E56" si="0">D23*10</f>
+        <f t="shared" ref="E23:E58" si="0">D23*10</f>
         <v>3.6691200000000004</v>
       </c>
       <c r="F23" s="131">
-        <f t="shared" ref="F23:F56" si="1">D23*50</f>
+        <f t="shared" ref="F23:F58" si="1">D23*50</f>
         <v>18.345600000000001</v>
       </c>
       <c r="G23" s="131">
-        <f t="shared" ref="G23:G56" si="2">D23*100</f>
+        <f t="shared" ref="G23:G58" si="2">D23*100</f>
         <v>36.691200000000002</v>
       </c>
       <c r="H23" s="131">
-        <f t="shared" ref="H23:H56" si="3">D23*500</f>
+        <f t="shared" ref="H23:H58" si="3">D23*500</f>
         <v>183.45600000000002</v>
       </c>
       <c r="I23" s="131">
-        <f t="shared" ref="I23:I56" si="4">D23*1000</f>
+        <f t="shared" ref="I23:I58" si="4">D23*1000</f>
         <v>366.91200000000003</v>
       </c>
     </row>
@@ -20946,68 +21120,68 @@
         <v>741.92666666666685</v>
       </c>
     </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B51" t="s">
+    <row r="51" spans="2:9" s="59" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="59" t="s">
         <v>61</v>
       </c>
-      <c r="C51">
-        <v>7</v>
+      <c r="C51" s="59">
+        <v>5</v>
       </c>
       <c r="D51" s="131">
-        <f>N17</f>
-        <v>0.78139999999999998</v>
+        <f t="shared" ref="D51:D53" si="5">N14*1.056</f>
+        <v>0.40360320000000005</v>
       </c>
       <c r="E51" s="131">
-        <f t="shared" si="0"/>
-        <v>7.8140000000000001</v>
+        <f t="shared" ref="E51:E53" si="6">D51*10</f>
+        <v>4.0360320000000005</v>
       </c>
       <c r="F51" s="131">
-        <f t="shared" si="1"/>
-        <v>39.07</v>
+        <f t="shared" ref="F51:F53" si="7">D51*50</f>
+        <v>20.180160000000001</v>
       </c>
       <c r="G51" s="131">
-        <f t="shared" si="2"/>
-        <v>78.14</v>
+        <f t="shared" ref="G51:G53" si="8">D51*100</f>
+        <v>40.360320000000002</v>
       </c>
       <c r="H51" s="131">
-        <f t="shared" si="3"/>
-        <v>390.7</v>
+        <f t="shared" ref="H51:H53" si="9">D51*500</f>
+        <v>201.80160000000004</v>
       </c>
       <c r="I51" s="131">
-        <f t="shared" si="4"/>
-        <v>781.4</v>
-      </c>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
+        <f t="shared" ref="I51:I53" si="10">D51*1000</f>
+        <v>403.60320000000007</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" s="59" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="59" t="s">
         <v>61</v>
       </c>
-      <c r="C52">
-        <v>8</v>
+      <c r="C52" s="59">
+        <v>6</v>
       </c>
       <c r="D52" s="131">
-        <f>N17*1.056</f>
-        <v>0.82515840000000007</v>
+        <f t="shared" si="5"/>
+        <v>0.44510400000000006</v>
       </c>
       <c r="E52" s="131">
-        <f t="shared" si="0"/>
-        <v>8.2515840000000011</v>
+        <f t="shared" si="6"/>
+        <v>4.4510400000000008</v>
       </c>
       <c r="F52" s="131">
-        <f t="shared" si="1"/>
-        <v>41.257920000000006</v>
+        <f t="shared" si="7"/>
+        <v>22.255200000000002</v>
       </c>
       <c r="G52" s="131">
-        <f t="shared" si="2"/>
-        <v>82.515840000000011</v>
+        <f t="shared" si="8"/>
+        <v>44.510400000000004</v>
       </c>
       <c r="H52" s="131">
-        <f t="shared" si="3"/>
-        <v>412.57920000000001</v>
+        <f t="shared" si="9"/>
+        <v>222.55200000000002</v>
       </c>
       <c r="I52" s="131">
-        <f t="shared" si="4"/>
-        <v>825.15840000000003</v>
+        <f t="shared" si="10"/>
+        <v>445.10400000000004</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
@@ -21015,31 +21189,31 @@
         <v>61</v>
       </c>
       <c r="C53">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D53" s="131">
-        <f>N17*1.112</f>
-        <v>0.86891680000000004</v>
+        <f t="shared" si="5"/>
+        <v>0.71878400000000009</v>
       </c>
       <c r="E53" s="131">
-        <f t="shared" si="0"/>
-        <v>8.6891680000000004</v>
+        <f t="shared" si="6"/>
+        <v>7.1878400000000013</v>
       </c>
       <c r="F53" s="131">
-        <f t="shared" si="1"/>
-        <v>43.445840000000004</v>
+        <f t="shared" si="7"/>
+        <v>35.939200000000007</v>
       </c>
       <c r="G53" s="131">
-        <f t="shared" si="2"/>
-        <v>86.891680000000008</v>
+        <f t="shared" si="8"/>
+        <v>71.878400000000013</v>
       </c>
       <c r="H53" s="131">
-        <f t="shared" si="3"/>
-        <v>434.45840000000004</v>
+        <f t="shared" si="9"/>
+        <v>359.39200000000005</v>
       </c>
       <c r="I53" s="131">
-        <f t="shared" si="4"/>
-        <v>868.91680000000008</v>
+        <f t="shared" si="10"/>
+        <v>718.78400000000011</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
@@ -21047,31 +21221,31 @@
         <v>61</v>
       </c>
       <c r="C54">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D54" s="131">
-        <f>N17*1.168</f>
-        <v>0.91267519999999991</v>
+        <f>N17*1.056</f>
+        <v>0.82515840000000007</v>
       </c>
       <c r="E54" s="131">
         <f t="shared" si="0"/>
-        <v>9.1267519999999998</v>
+        <v>8.2515840000000011</v>
       </c>
       <c r="F54" s="131">
         <f t="shared" si="1"/>
-        <v>45.633759999999995</v>
+        <v>41.257920000000006</v>
       </c>
       <c r="G54" s="131">
         <f t="shared" si="2"/>
-        <v>91.26751999999999</v>
+        <v>82.515840000000011</v>
       </c>
       <c r="H54" s="131">
         <f t="shared" si="3"/>
-        <v>456.33759999999995</v>
+        <v>412.57920000000001</v>
       </c>
       <c r="I54" s="131">
         <f t="shared" si="4"/>
-        <v>912.6751999999999</v>
+        <v>825.15840000000003</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
@@ -21079,31 +21253,31 @@
         <v>61</v>
       </c>
       <c r="C55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D55" s="131">
-        <f>N17*1.224</f>
-        <v>0.95643359999999999</v>
+        <f>N17*1.112</f>
+        <v>0.86891680000000004</v>
       </c>
       <c r="E55" s="131">
         <f t="shared" si="0"/>
-        <v>9.5643360000000008</v>
+        <v>8.6891680000000004</v>
       </c>
       <c r="F55" s="131">
         <f t="shared" si="1"/>
-        <v>47.821680000000001</v>
+        <v>43.445840000000004</v>
       </c>
       <c r="G55" s="131">
         <f t="shared" si="2"/>
-        <v>95.643360000000001</v>
+        <v>86.891680000000008</v>
       </c>
       <c r="H55" s="131">
         <f t="shared" si="3"/>
-        <v>478.21679999999998</v>
+        <v>434.45840000000004</v>
       </c>
       <c r="I55" s="131">
         <f t="shared" si="4"/>
-        <v>956.43359999999996</v>
+        <v>868.91680000000008</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
@@ -21111,35 +21285,124 @@
         <v>61</v>
       </c>
       <c r="C56">
+        <v>10</v>
+      </c>
+      <c r="D56" s="131">
+        <f>N17*1.168</f>
+        <v>0.91267519999999991</v>
+      </c>
+      <c r="E56" s="131">
+        <f t="shared" si="0"/>
+        <v>9.1267519999999998</v>
+      </c>
+      <c r="F56" s="131">
+        <f t="shared" si="1"/>
+        <v>45.633759999999995</v>
+      </c>
+      <c r="G56" s="131">
+        <f t="shared" si="2"/>
+        <v>91.26751999999999</v>
+      </c>
+      <c r="H56" s="131">
+        <f t="shared" si="3"/>
+        <v>456.33759999999995</v>
+      </c>
+      <c r="I56" s="131">
+        <f t="shared" si="4"/>
+        <v>912.6751999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>61</v>
+      </c>
+      <c r="C57">
+        <v>11</v>
+      </c>
+      <c r="D57" s="131">
+        <f>N17*1.224</f>
+        <v>0.95643359999999999</v>
+      </c>
+      <c r="E57" s="131">
+        <f t="shared" si="0"/>
+        <v>9.5643360000000008</v>
+      </c>
+      <c r="F57" s="131">
+        <f t="shared" si="1"/>
+        <v>47.821680000000001</v>
+      </c>
+      <c r="G57" s="131">
+        <f t="shared" si="2"/>
+        <v>95.643360000000001</v>
+      </c>
+      <c r="H57" s="131">
+        <f t="shared" si="3"/>
+        <v>478.21679999999998</v>
+      </c>
+      <c r="I57" s="131">
+        <f t="shared" si="4"/>
+        <v>956.43359999999996</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58">
         <v>12</v>
       </c>
-      <c r="D56" s="131">
+      <c r="D58" s="131">
         <f>N17*1.28</f>
         <v>1.000192</v>
       </c>
-      <c r="E56" s="131">
+      <c r="E58" s="131">
         <f t="shared" si="0"/>
         <v>10.00192</v>
       </c>
-      <c r="F56" s="131">
+      <c r="F58" s="131">
         <f t="shared" si="1"/>
         <v>50.009599999999999</v>
       </c>
-      <c r="G56" s="131">
+      <c r="G58" s="131">
         <f t="shared" si="2"/>
         <v>100.0192</v>
       </c>
-      <c r="H56" s="131">
+      <c r="H58" s="131">
         <f t="shared" si="3"/>
         <v>500.096</v>
       </c>
-      <c r="I56" s="131">
+      <c r="I58" s="131">
         <f t="shared" si="4"/>
         <v>1000.192</v>
       </c>
     </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B59" s="59" t="s">
+        <v>383</v>
+      </c>
+      <c r="C59" s="59">
+        <v>16</v>
+      </c>
+      <c r="D59" s="131">
+        <f>$N$18*1.28</f>
+        <v>6.8838400000000002</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B60" s="59" t="s">
+        <v>383</v>
+      </c>
+      <c r="C60" s="59">
+        <v>17</v>
+      </c>
+      <c r="D60" s="131">
+        <f>$N$18*1.28</f>
+        <v>6.8838400000000002</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="N18:O18"/>
     <mergeCell ref="N17:O17"/>
     <mergeCell ref="N15:O15"/>
     <mergeCell ref="N16:O16"/>

</xml_diff>